<commit_message>
Extract RA2CE road-preprocessing chain; fix test-graph hazard alignment
- Add book/preprocessing/prep_data_from_extent.py, isolating just the
  road/RA2CE build-and-hazard-overlay chain from
  prep_data_from_rasterextent.ipynb (network extent, RA2CE run, hazard-column
  zero-padding, blank-raster fill for the recovery period). Electricity-asset
  work is intentionally excluded, it duplicates existing loaders.
- Regenerate data/test_samples/static/{network,output_graph}/* so EV{n}_ma on
  base_graph_hazard_editted.p correctly matches Frag_timesteps_test{n}.tif
  (previously the test graph's hazard columns were unrelated to this raster
  series, so the flooded band never fragmented the network).
- Ignore local _backup snapshots under output_graph/.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/test_samples/static/output_graph/hazard_names.xlsx
+++ b/data/test_samples/static/output_graph/hazard_names.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test1.tif</t>
+          <t>C:\repos\powerpath-societal-access\data\test_samples\test_hazard_timesteps\Frag_timesteps_test1.tif</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test1.tif</t>
+          <t>C:\repos\powerpath-societal-access\data\test_samples\test_hazard_timesteps\Frag_timesteps_test1.tif</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test2.tif</t>
+          <t>C:\repos\powerpath-societal-access\data\test_samples\test_hazard_timesteps\Frag_timesteps_test2.tif</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test2.tif</t>
+          <t>C:\repos\powerpath-societal-access\data\test_samples\test_hazard_timesteps\Frag_timesteps_test2.tif</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test3.tif</t>
+          <t>C:\repos\powerpath-societal-access\data\test_samples\test_hazard_timesteps\Frag_timesteps_test3.tif</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test3.tif</t>
+          <t>C:\repos\powerpath-societal-access\data\test_samples\test_hazard_timesteps\Frag_timesteps_test3.tif</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test4.tif</t>
+          <t>C:\repos\powerpath-societal-access\data\test_samples\test_hazard_timesteps\Frag_timesteps_test4.tif</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test4.tif</t>
+          <t>C:\repos\powerpath-societal-access\data\test_samples\test_hazard_timesteps\Frag_timesteps_test4.tif</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test5.tif</t>
+          <t>C:\repos\powerpath-societal-access\data\test_samples\test_hazard_timesteps\Frag_timesteps_test5.tif</t>
         </is>
       </c>
     </row>
@@ -666,183 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test5.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Frag_timesteps_test6</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>maximum</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>EV6_ma</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test6.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Frag_timesteps_test6</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>fraction of network segment impacted by hazard</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>EV6_fr</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test6.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Frag_timesteps_test7</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>maximum</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>EV7_ma</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test7.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Frag_timesteps_test7</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>fraction of network segment impacted by hazard</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>EV7_fr</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test7.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Frag_timesteps_test8</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>maximum</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>EV8_ma</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test8.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Frag_timesteps_test8</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>fraction of network segment impacted by hazard</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>EV8_fr</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test8.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Frag_timesteps_test9</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>maximum</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>EV9_ma</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test9.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Frag_timesteps_test9</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>fraction of network segment impacted by hazard</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>EV9_fr</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test9.tif</t>
+          <t>C:\repos\powerpath-societal-access\data\test_samples\test_hazard_timesteps\Frag_timesteps_test5.tif</t>
         </is>
       </c>
     </row>

</xml_diff>